<commit_message>
Initial commit - CCTV surveillance system
</commit_message>
<xml_diff>
--- a/attendance_master.xlsx
+++ b/attendance_master.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,8 +30,16 @@
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <color rgb="0078550A"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <color rgb="00065F46"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +49,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E6F9F0"/>
       </patternFill>
     </fill>
   </fills>
@@ -62,9 +80,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -432,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -481,6 +505,916 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>19:44:05</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>19:53:32</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>19:53:44</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>00:00:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>19:53:52</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>19:53:58</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>00:00:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>19:54:35</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>19:55:09</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>00:00:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>19:55:18</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>19:55:24</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>00:00:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>19:56:13</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>19:57:02</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>00:00:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>19:58:01</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>19:58:15</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>00:00:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>19:58:27</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>19:58:35</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>00:00:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>19:59:34</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>19:59:44</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>00:00:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>20:00:59</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>20:02:23</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>00:01:24</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>20:02:53</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>20:09:59</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>20:10:34</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>00:00:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>20:10:35</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>20:10:49</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>00:00:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>20:11:44</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>20:13:02</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>00:01:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>20:15:01</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>20:15:30</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>00:00:29</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>20:15:39</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>20:16:51</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>00:01:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>21:09:48</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>21:10:03</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>00:00:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>21:10:29</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>21:10:45</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>00:00:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>21:11:02</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>21:11:09</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>00:00:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>21:11:18</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>21:12:16</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>00:00:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>4CSM-2</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>21:12:18</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>21:13:43</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>21:14:05</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>00:00:22</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>21:14:08</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>21:14:22</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>00:00:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>21:14:29</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>21:14:35</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>00:00:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>21:59:11</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Vaghdevi</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>322103282073</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>28-02-2026</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>22:16:38</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>